<commit_message>
Fix small layout issues
</commit_message>
<xml_diff>
--- a/TelemDefinition/DownlinkSpecPacsat.xlsx
+++ b/TelemDefinition/DownlinkSpecPacsat.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chris\workspace_ccs\PacSatDocs\TelemDefinition\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F39A7465-62B4-408A-B2D1-18FF48D9786C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FC1F0C0-A01E-4884-8DFC-76BB2AD56780}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="24105" windowHeight="13920" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="26310" windowHeight="13920" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DownlinkSpecPacsat" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="799" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="799" uniqueCount="347">
   <si>
     <t>//</t>
   </si>
@@ -1072,6 +1072,12 @@
   </si>
   <si>
     <t>Time to Downlink</t>
+  </si>
+  <si>
+    <t>Pwr Mode</t>
+  </si>
+  <si>
+    <t>RSSI</t>
   </si>
 </sst>
 </file>
@@ -2462,7 +2468,7 @@
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B26" s="20" t="s">
-        <v>68</v>
+        <v>345</v>
       </c>
       <c r="C26" s="20" t="s">
         <v>68</v>
@@ -2558,7 +2564,7 @@
         <v>4</v>
       </c>
       <c r="P27" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q27" s="1">
         <v>0</v>
@@ -2566,7 +2572,7 @@
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B28" s="20" t="s">
-        <v>73</v>
+        <v>345</v>
       </c>
       <c r="C28" s="20" t="s">
         <v>73</v>
@@ -2618,7 +2624,7 @@
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B29" s="20" t="s">
-        <v>76</v>
+        <v>345</v>
       </c>
       <c r="C29" s="20" t="s">
         <v>76</v>
@@ -2670,7 +2676,7 @@
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
-        <v>79</v>
+        <v>345</v>
       </c>
       <c r="C30" s="20" t="s">
         <v>79</v>
@@ -2722,7 +2728,7 @@
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B31" s="20" t="s">
-        <v>82</v>
+        <v>345</v>
       </c>
       <c r="C31" s="20" t="s">
         <v>82</v>
@@ -2982,7 +2988,7 @@
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B36" s="20" t="s">
-        <v>93</v>
+        <v>346</v>
       </c>
       <c r="C36" s="20" t="s">
         <v>93</v>
@@ -3034,7 +3040,7 @@
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B37" s="20" t="s">
-        <v>96</v>
+        <v>346</v>
       </c>
       <c r="C37" s="20" t="s">
         <v>96</v>
@@ -3086,7 +3092,7 @@
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B38" s="20" t="s">
-        <v>98</v>
+        <v>346</v>
       </c>
       <c r="C38" s="20" t="s">
         <v>98</v>
@@ -3138,7 +3144,7 @@
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.2">
       <c r="B39" s="20" t="s">
-        <v>100</v>
+        <v>346</v>
       </c>
       <c r="C39" s="20" t="s">
         <v>100</v>
@@ -3338,7 +3344,7 @@
         <v>2</v>
       </c>
       <c r="P42" s="1">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="Q42" s="1">
         <v>0</v>
@@ -5778,7 +5784,7 @@
         <v>1</v>
       </c>
       <c r="P107" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q107" s="1">
         <v>0</v>
@@ -5830,7 +5836,7 @@
         <v>1</v>
       </c>
       <c r="P108" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q108" s="1">
         <v>0</v>
@@ -5882,7 +5888,7 @@
         <v>1</v>
       </c>
       <c r="P109" s="1">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q109" s="1">
         <v>0</v>

</xml_diff>

<commit_message>
Fix formatting of board voltages
</commit_message>
<xml_diff>
--- a/TelemDefinition/DownlinkSpecPacsat.xlsx
+++ b/TelemDefinition/DownlinkSpecPacsat.xlsx
@@ -377,7 +377,7 @@
     <t xml:space="preserve">VoltageVal3v3</t>
   </si>
   <si>
-    <t xml:space="preserve">V</t>
+    <t xml:space="preserve">mV</t>
   </si>
   <si>
     <t xml:space="preserve">Voltage of the 3V3 rail</t>
@@ -3208,7 +3208,7 @@
       </c>
       <c r="F43" s="19"/>
       <c r="G43" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H43" s="18" t="s">
         <v>118</v>
@@ -3260,7 +3260,7 @@
       </c>
       <c r="F44" s="19"/>
       <c r="G44" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H44" s="18" t="s">
         <v>118</v>
@@ -3312,7 +3312,7 @@
       </c>
       <c r="F45" s="19"/>
       <c r="G45" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H45" s="18" t="s">
         <v>118</v>
@@ -3364,7 +3364,7 @@
       </c>
       <c r="F46" s="19"/>
       <c r="G46" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H46" s="18" t="s">
         <v>118</v>
@@ -9006,7 +9006,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B6:I20"/>
-  <sheetFormatPr defaultColWidth="9.31640625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.328125" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16.14"/>

</xml_diff>